<commit_message>
I created a function that allows for the assignments to be saved to the actual excel file once they are submitted. I made sure to call this function inside of the submit function.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/assignments.xlsx
+++ b/assignments.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -40,6 +40,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004ECBA1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF6B6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -55,9 +65,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -425,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -468,6 +484,98 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Smartbook</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>4/27/2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Chapter 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Application Development</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>4/29/2026</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>CHapter 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Information Systems</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>5/1/2026</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
I have created a function that allows me to load assignments that have already been uploaded to the excel file to the application as it is opened.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/assignments.xlsx
+++ b/assignments.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +52,11 @@
         <fgColor rgb="00FF6B6B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5A623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -74,6 +79,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -441,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -576,6 +584,38 @@
       </c>
       <c r="F4" s="3" t="inlineStr"/>
     </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Honors</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Chapter 6</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
In this code I created a delete button and a delete function to allow the user to delete a current assignment from the listbox and excel worksheet.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/assignments.xlsx
+++ b/assignments.xlsx
@@ -1,104 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kennesawedu-my.sharepoint.com/personal/bturn116_students_kennesaw_edu/Documents/Task-Assignment-Tracker/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_685E3F77157CC0DEE75BECD44CD28E3A95F6C1AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC3A57A4-FBD2-1348-A4C2-722791E78E17}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Assignments" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Assignments!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assignments'!$A$1:$F$3</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
-  <si>
-    <t>Assignment Name</t>
-  </si>
-  <si>
-    <t>Class</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Due Date</t>
-  </si>
-  <si>
-    <t>Priority</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Smartbook</t>
-  </si>
-  <si>
-    <t>Accounting</t>
-  </si>
-  <si>
-    <t>Homework</t>
-  </si>
-  <si>
-    <t>4/26/2026</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Chapter 22</t>
-  </si>
-  <si>
-    <t>Quiz</t>
-  </si>
-  <si>
-    <t>Management</t>
-  </si>
-  <si>
-    <t>05/01/2026</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Chapter 12</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -132,30 +70,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -443,79 +440,87 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="25" customWidth="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Assignment Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Due Date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>16</v>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Smartbook</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Accounting</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>4/26/2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Chapter 22</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F3">
+  <autoFilter ref="A1:F3">
+    <sortState ref="A2:F3">
       <sortCondition ref="E1:E3"/>
     </sortState>
   </autoFilter>

</xml_diff>

<commit_message>
I created a target date function which allows the user to include a target date if they would like to. This would be the date they plan to get the assignment done by.
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/assignments.xlsx
+++ b/assignments.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assignments" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assignments'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assignments'!$A$1:$G$1</definedName>
   </definedNames>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -27,11 +28,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="5">
@@ -43,17 +41,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
+        <fgColor rgb="004472C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4ECBA1"/>
+        <fgColor rgb="004ECBA1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5A623"/>
+        <fgColor rgb="00F5A623"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,7 +80,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -445,13 +443,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,10 +478,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Target Date</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -489,41 +495,71 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Smartbook</t>
+          <t>smartbook</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>management</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Homework</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>05/02/2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>05/01/2026</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Chapter 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
           <t>Accounting</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Homework</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>4/26/2026</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Chapter 22</t>
-        </is>
-      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>4/30/2026</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3">
-    <sortState ref="A2:F3">
-      <sortCondition ref="E1:E3"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>